<commit_message>
Clean up metrics computaion
</commit_message>
<xml_diff>
--- a/code/data_management/meta_data_processing.xlsx
+++ b/code/data_management/meta_data_processing.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://alleninstitute-my.sharepoint.com/personal/sue_su_alleninstitute_org/Documents/LCpaper/manuscript/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="207" documentId="8_{13714737-15D5-6D46-9EE3-176A3926FE2A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{0FF5906D-7507-4880-89EB-C2944D6EC385}"/>
+  <xr:revisionPtr revIDLastSave="213" documentId="8_{13714737-15D5-6D46-9EE3-176A3926FE2A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{C3116327-9C4B-40E6-B1C9-03F8311B8F1D}"/>
   <bookViews>
     <workbookView xWindow="-28920" yWindow="7125" windowWidth="29040" windowHeight="15720" xr2:uid="{FFE2B52C-1751-7945-8601-5DA37AD336B9}"/>
   </bookViews>
@@ -41,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="87" uniqueCount="56">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="91" uniqueCount="59">
   <si>
     <t>name</t>
   </si>
@@ -209,6 +209,15 @@
   </si>
   <si>
     <t>code/beh_ephys_analysis/antidromic_funcs.py/analyze_antidromic_responses</t>
+  </si>
+  <si>
+    <t>compute_behavior_metrics</t>
+  </si>
+  <si>
+    <t>behavior/{session_id}_beh_metrics.json</t>
+  </si>
+  <si>
+    <t>code/beh_ephys_analysis/beh_metrics.py</t>
   </si>
 </sst>
 </file>
@@ -296,7 +305,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="12">
+  <cellXfs count="14">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -325,6 +334,12 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="1"/>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -855,7 +870,20 @@
         <v>28</v>
       </c>
     </row>
-    <row r="13" spans="1:5" ht="50" customHeight="1" x14ac:dyDescent="0.5"/>
+    <row r="13" spans="1:5" ht="50" customHeight="1" x14ac:dyDescent="0.7">
+      <c r="A13" s="12" t="s">
+        <v>56</v>
+      </c>
+      <c r="B13" s="13" t="s">
+        <v>57</v>
+      </c>
+      <c r="D13" s="7" t="s">
+        <v>14</v>
+      </c>
+      <c r="E13" s="2" t="s">
+        <v>58</v>
+      </c>
+    </row>
     <row r="14" spans="1:5" ht="50" customHeight="1" x14ac:dyDescent="0.5"/>
   </sheetData>
   <hyperlinks>
@@ -864,8 +892,10 @@
     <hyperlink ref="E9" r:id="rId3" display="https://github.com/AllenNeuralDynamics/aind-beh-ephys-analysis/blob/main/code/beh_ephys_analysis/ccf_generation.py/make_ccf_tbl" xr:uid="{86200356-EB70-DF4F-8FEA-70F94BCA000B}"/>
     <hyperlink ref="D12" r:id="rId4" xr:uid="{B0B15AFD-795D-BB42-94D1-7DB297F4B456}"/>
     <hyperlink ref="D3" r:id="rId5" xr:uid="{7D29D876-4DBD-834B-A286-6B3C96D33384}"/>
+    <hyperlink ref="D13" r:id="rId6" xr:uid="{E9017DD4-36DD-4F45-BB17-7B59F59BC27A}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId7"/>
 </worksheet>
 </file>
 

</xml_diff>